<commit_message>
feat: adding new feat
</commit_message>
<xml_diff>
--- a/sample_assets/sample_5_videos.xlsx
+++ b/sample_assets/sample_5_videos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH6"/>
+  <dimension ref="A1:AI6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -587,6 +587,11 @@
           <t>CTA_Video_Fade_Duration</t>
         </is>
       </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>CTA_Video_Speed</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -708,6 +713,9 @@
       </c>
       <c r="AH2" t="n">
         <v>0.8</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -811,6 +819,9 @@
       <c r="AH3" t="n">
         <v>0.4</v>
       </c>
+      <c r="AI3" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr"/>
@@ -920,6 +931,9 @@
       </c>
       <c r="AH4" t="n">
         <v>0.5</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -969,6 +983,7 @@
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
       <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr"/>
@@ -1041,6 +1056,7 @@
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
       <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>